<commit_message>
qa: max verify — Phase 1 + Phase 2 all cases pass on Railway
Bulk-flip: 28 pending cases → pass ("Verified on Railway"). Covers:
  - Phase 1 Dedup & signatory group (CI-59..64) — same-doc/two-phone
    scenario played end-to-end; CI-61's reported "appointment gone
    after convert-to-petition" bug confirmed fixed.
  - Phase 2 (PR-01..22) — full Petition Review sweep on /ai-review:
    RBAC, list/filters, drawer content, triage (approve/dismiss/
    restore), edits, attachments, signatory merge, comments, UX.

Two intentional skips stay skipped:
  - CI-23  rate limit (RATE_LIMIT_ENABLED=false globally in test env)
  - CI-71  one-per-day guard ON (ONE_PETITION_PER_DAY=false in test env)

Totals: 113 · 111 pass · 2 skipped · 0 pending.

Header comment cleaned — the "except dedup" note is now stale.
META.gitSha bumped to 3f0df68 (matches the last pill-count parity fix
that landed in this arc).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa/test-cases.xlsx
+++ b/qa/test-cases.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,12 +53,8 @@
       <b val="1"/>
       <color rgb="005B21B6"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00374151"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -78,11 +74,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EDE9FE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E5E7EB"/>
       </patternFill>
     </fill>
   </fills>
@@ -112,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -127,9 +118,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -543,7 +531,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4a26213</t>
+          <t>3f0df68</t>
         </is>
       </c>
     </row>
@@ -595,7 +583,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -615,7 +603,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>83</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15">
@@ -655,7 +643,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>85</v>
+        <v>113</v>
       </c>
     </row>
     <row r="19">
@@ -666,7 +654,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -3383,12 +3371,16 @@
           <t>Two independent tickets, both AWAITING_REVIEW; both appointments visible</t>
         </is>
       </c>
-      <c r="G60" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H60" s="5" t="inlineStr"/>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
           <t>Setup for CI-60/61. Awaiting focused end-to-end pass — reported-bug regression.</t>
@@ -3427,12 +3419,16 @@
           <t>Petition row created; A's appointment still linked; ticket advances</t>
         </is>
       </c>
-      <c r="G61" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H61" s="5" t="inlineStr"/>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I61" s="5" t="inlineStr"/>
     </row>
     <row r="62" ht="60" customHeight="1">
@@ -3467,12 +3463,16 @@
           <t>Either merges into A's signatory list WITH B's appointment PRESERVED, OR creates B as separate petition. B's appointment must not vanish.</t>
         </is>
       </c>
-      <c r="G62" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H62" s="5" t="inlineStr"/>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
           <t>USER-REPORTED BUG: 'appointment gone and not found in the petition too'. Focus of the dedup pass.</t>
@@ -3511,12 +3511,16 @@
           <t>Second recognized as same citizen (mobile blind index match); either updates name or flags conflict; no duplicate citizen row</t>
         </is>
       </c>
-      <c r="G63" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H63" s="5" t="inlineStr"/>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
           <t>Verifies Fernet encryption + SHA-256 blind index</t>
@@ -3555,12 +3559,16 @@
           <t>Recognized as same citizen; name normalization consistent</t>
         </is>
       </c>
-      <c r="G64" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H64" s="5" t="inlineStr"/>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I64" s="5" t="inlineStr"/>
     </row>
     <row r="65" ht="60" customHeight="1">
@@ -3595,12 +3603,16 @@
           <t>Both persisted OR one wins with clean dedup; no orphan rows, no partial state, no double-commit</t>
         </is>
       </c>
-      <c r="G65" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H65" s="5" t="inlineStr"/>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I65" s="5" t="inlineStr">
         <is>
           <t>Verifies CORR-06 signatory merge FOR UPDATE row-lock</t>
@@ -4896,12 +4908,16 @@
           <t>pa_admin sees the list. dept_officer redirected to /tickets (per _no_dept_officer gate).</t>
         </is>
       </c>
-      <c r="G93" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H93" s="5" t="inlineStr"/>
+      <c r="G93" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I93" s="5" t="inlineStr"/>
     </row>
     <row r="94" ht="60" customHeight="1">
@@ -4936,12 +4952,16 @@
           <t>302 to /auth/login; no traceback; no data leaked</t>
         </is>
       </c>
-      <c r="G94" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H94" s="5" t="inlineStr"/>
+      <c r="G94" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H94" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I94" s="5" t="inlineStr"/>
     </row>
     <row r="95" ht="60" customHeight="1">
@@ -4976,12 +4996,16 @@
           <t>Only AWAITING_REVIEW rows appear. Empty-state is friendly when count is zero.</t>
         </is>
       </c>
-      <c r="G95" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H95" s="5" t="inlineStr"/>
+      <c r="G95" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H95" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I95" s="5" t="inlineStr"/>
     </row>
     <row r="96" ht="60" customHeight="1">
@@ -5017,12 +5041,16 @@
           <t>Each control narrows the list correctly. Newest-first default has an id tie-break (PERF-08). Clear-all restores.</t>
         </is>
       </c>
-      <c r="G96" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H96" s="5" t="inlineStr"/>
+      <c r="G96" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H96" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I96" s="5" t="inlineStr"/>
     </row>
     <row r="97" ht="60" customHeight="1">
@@ -5058,12 +5086,16 @@
           <t>Page 2 shows next 25 (no dupes). Counts match exactly (no IST/UTC drift). Fresh submission appears after the polling interval.</t>
         </is>
       </c>
-      <c r="G97" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H97" s="5" t="inlineStr"/>
+      <c r="G97" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H97" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I97" s="5" t="inlineStr"/>
     </row>
     <row r="98" ht="60" customHeight="1">
@@ -5099,12 +5131,16 @@
           <t>Both entry points open the drawer with the right row. X and Esc close it. Browser back closes it too.</t>
         </is>
       </c>
-      <c r="G98" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H98" s="5" t="inlineStr"/>
+      <c r="G98" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H98" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I98" s="5" t="inlineStr"/>
     </row>
     <row r="99" ht="60" customHeight="1">
@@ -5139,12 +5175,16 @@
           <t>Name / masked mobile (******3210) / constituency / district present. Category + priority (colour-coded) + ministry pills reflect GSR.</t>
         </is>
       </c>
-      <c r="G99" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H99" s="5" t="inlineStr"/>
+      <c r="G99" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H99" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I99" s="5" t="inlineStr">
         <is>
           <t>Mobile mask regression</t>
@@ -5183,12 +5223,16 @@
           <t>Tamil renders in Noto Serif Tamil, English in Inter. No ???. Bullets render as bullets.</t>
         </is>
       </c>
-      <c r="G100" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H100" s="5" t="inlineStr"/>
+      <c r="G100" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H100" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I100" s="5" t="inlineStr"/>
     </row>
     <row r="101" ht="60" customHeight="1">
@@ -5223,12 +5267,16 @@
           <t>PDF iframe: XFO SAMEORIGIN + frame-ancestors 'self' honoured (CI-89 regression). Audio: Range requests supported, seek works, duration finite on WebM/Opus.</t>
         </is>
       </c>
-      <c r="G101" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H101" s="5" t="inlineStr"/>
+      <c r="G101" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H101" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I101" s="5" t="inlineStr">
         <is>
           <t>CI-89 iframe fix regression, PERF-audio Range</t>
@@ -5268,12 +5316,16 @@
           <t>New Ticket with correct ticket_number (TKN&lt;year&gt;&lt;ord&gt;), status=OPEN, appointment_id linked. Appt.status → REVIEWED. Row leaves the AWAITING_REVIEW list.</t>
         </is>
       </c>
-      <c r="G102" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H102" s="5" t="inlineStr"/>
+      <c r="G102" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H102" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I102" s="5" t="inlineStr"/>
     </row>
     <row r="103" ht="60" customHeight="1">
@@ -5309,12 +5361,16 @@
           <t>spawn_bg(_notify) log line present. Activity row: action_type='created', user='pa_admin', payload has {token, appointment_id}.</t>
         </is>
       </c>
-      <c r="G103" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H103" s="5" t="inlineStr"/>
+      <c r="G103" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H103" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I103" s="5" t="inlineStr"/>
     </row>
     <row r="104" ht="60" customHeight="1">
@@ -5349,12 +5405,16 @@
           <t>One ticket only. Button disabled during in-flight submit. No 500.</t>
         </is>
       </c>
-      <c r="G104" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H104" s="5" t="inlineStr"/>
+      <c r="G104" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H104" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I104" s="5" t="inlineStr"/>
     </row>
     <row r="105" ht="60" customHeight="1">
@@ -5391,12 +5451,16 @@
           <t>Status transitions cleanly both ways. Activity log records dismiss (with reason) + restore.</t>
         </is>
       </c>
-      <c r="G105" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H105" s="5" t="inlineStr"/>
+      <c r="G105" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H105" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I105" s="5" t="inlineStr"/>
     </row>
     <row r="106" ht="60" customHeight="1">
@@ -5431,12 +5495,16 @@
           <t>PATCH /details persists. Name update rehashes the blind-index. AI-inferred values overridden on save. No silent 500 on two-tab conflict — either overwrites cleanly or shows a 'refresh' message.</t>
         </is>
       </c>
-      <c r="G106" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H106" s="5" t="inlineStr"/>
+      <c r="G106" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H106" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I106" s="5" t="inlineStr"/>
     </row>
     <row r="107" ht="60" customHeight="1">
@@ -5472,12 +5540,16 @@
           <t>Uploads succeed and preview inline. 5MB size cap + 10-file total cap enforced with a clean human message.</t>
         </is>
       </c>
-      <c r="G107" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H107" s="5" t="inlineStr"/>
+      <c r="G107" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H107" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I107" s="5" t="inlineStr"/>
     </row>
     <row r="108" ht="60" customHeight="1">
@@ -5512,12 +5584,16 @@
           <t>Filename escaped everywhere. No alert dialog. No console error.</t>
         </is>
       </c>
-      <c r="G108" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H108" s="5" t="inlineStr"/>
+      <c r="G108" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H108" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I108" s="5" t="inlineStr">
         <is>
           <t>CITZ-02 regression via drawer surface</t>
@@ -5556,12 +5632,16 @@
           <t>Similar list is category+district-blocked and similarity-scored. Merge attaches current appt as signatory of target; no new Ticket row.</t>
         </is>
       </c>
-      <c r="G109" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H109" s="5" t="inlineStr"/>
+      <c r="G109" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H109" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I109" s="5" t="inlineStr"/>
     </row>
     <row r="110" ht="60" customHeight="1">
@@ -5597,12 +5677,16 @@
           <t>Neither appointment disappears. The reported bug 'appointment gone after convert' stays fixed via the merge path too.</t>
         </is>
       </c>
-      <c r="G110" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H110" s="5" t="inlineStr"/>
+      <c r="G110" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H110" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I110" s="5" t="inlineStr">
         <is>
           <t>PRIMARY dedup regression check</t>
@@ -5641,12 +5725,16 @@
           <t>One wins. The other gets a clean 'already merged' message. No duplicate signatory row. No partial state.</t>
         </is>
       </c>
-      <c r="G111" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H111" s="5" t="inlineStr"/>
+      <c r="G111" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H111" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I111" s="5" t="inlineStr">
         <is>
           <t>CORR-06 FOR UPDATE lock</t>
@@ -5685,12 +5773,16 @@
           <t>Both persist. Both render correctly in the activity feed (no ???, no codec err — the comment path is DB-only, not Gemini).</t>
         </is>
       </c>
-      <c r="G112" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H112" s="5" t="inlineStr"/>
+      <c r="G112" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H112" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I112" s="5" t="inlineStr"/>
     </row>
     <row r="113" ht="60" customHeight="1">
@@ -5725,12 +5817,16 @@
           <t>Every message is user-friendly. Zero tracebacks / 'gemini-2.5-flash' / raw HTTP codes. Routed through businessMessage() (errors.ts).</t>
         </is>
       </c>
-      <c r="G113" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H113" s="5" t="inlineStr"/>
+      <c r="G113" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I113" s="5" t="inlineStr"/>
     </row>
     <row r="114" ht="60" customHeight="1">
@@ -5765,12 +5861,16 @@
           <t>Drawer scales / becomes a full-screen sheet. All actions reachable. No horizontal body scroll.</t>
         </is>
       </c>
-      <c r="G114" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H114" s="5" t="inlineStr"/>
+      <c r="G114" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H114" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I114" s="5" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
qa: Phase 3 verified — all 20 Tickets + Association Review cases pass
User confirmed on Railway: "tested phase 3 cases, working fine".

Flipped every P3 case pending → pass with "Verified on Railway":
  TK-01..TK-11  (11 tickets cases)
  AR-01..AR-07  (7 association-review cases)
  T3-01, T3-02  (2 cross-cutting)

Regressions specifically covered stayed green under the sweep:
  TK-03  pill-count parity (3f0df68)
  TK-05  Assign only needs dept (2d1ee54)
  TK-06  Priority + due-date live-save on non-OPEN (decc4f4)
  TK-08  Filename XSS from ticket drawer (CITZ-02)
  TK-09  Dept ai_uploads/ PDF access (cbc9c8c + f40c2f6)
  TK-11  Drawer prev/next (5c3bc5b)
  AR-04  Ministry-driven decision (40a6f55)
  AR-05  Non-school auto-forward chain

Totals: 150 · 131 pass · 17 pending (Phase 4 only) · 2 skipped.
META.gitSha bumped to daa51f8.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa/test-cases.xlsx
+++ b/qa/test-cases.xlsx
@@ -543,7 +543,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3f0df68</t>
+          <t>daa51f8</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>37</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>111</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>113</v>
+        <v>133</v>
       </c>
     </row>
     <row r="19">
@@ -666,7 +666,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>88%</t>
         </is>
       </c>
     </row>
@@ -5917,12 +5917,16 @@
           <t>pa_admin: full ticket list across every dept. dept_officer: only tickets routed to their department; other rows never surface.</t>
         </is>
       </c>
-      <c r="G115" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H115" s="5" t="inlineStr"/>
+      <c r="G115" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H115" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I115" s="5" t="inlineStr"/>
     </row>
     <row r="116" ht="60" customHeight="1">
@@ -5957,12 +5961,16 @@
           <t>Each tab shows only its status. Rows never appear on the wrong tab. Terminal tabs (Resolved/Closed) don't show OPEN or FORWARDED rows.</t>
         </is>
       </c>
-      <c r="G116" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H116" s="5" t="inlineStr"/>
+      <c r="G116" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H116" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I116" s="5" t="inlineStr"/>
     </row>
     <row r="117" ht="60" customHeight="1">
@@ -5998,12 +6006,16 @@
           <t>Pill counts = visible list count for the same tab (no stable-universe mismatch). SLA-breached chip also narrows with the filter (already WYSIWYG per 0cde4ed).</t>
         </is>
       </c>
-      <c r="G117" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H117" s="5" t="inlineStr"/>
+      <c r="G117" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H117" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I117" s="5" t="inlineStr">
         <is>
           <t>Regression for 3f0df68 pill-count parity (aligns tickets with appointments + ai-review)</t>
@@ -6042,12 +6054,16 @@
           <t>Citizen tickets show petition summary + key details. Association tickets additionally show source_kind='association' detail card (a4bacc9).</t>
         </is>
       </c>
-      <c r="G118" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H118" s="5" t="inlineStr"/>
+      <c r="G118" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H118" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I118" s="5" t="inlineStr"/>
     </row>
     <row r="119" ht="60" customHeight="1">
@@ -6083,12 +6099,16 @@
           <t>Assign button enables as soon as a dept is picked. Save routes to dept + logs 'routed'. Previous bug: button stayed disabled without a due-date.</t>
         </is>
       </c>
-      <c r="G119" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H119" s="5" t="inlineStr"/>
+      <c r="G119" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H119" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I119" s="5" t="inlineStr"/>
     </row>
     <row r="120" ht="60" customHeight="1">
@@ -6124,12 +6144,16 @@
           <t>Both fields save immediately (canEditSla path). Prior bug: everything was disabled because canEdit gated on status===open.</t>
         </is>
       </c>
-      <c r="G120" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H120" s="5" t="inlineStr"/>
+      <c r="G120" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H120" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I120" s="5" t="inlineStr">
         <is>
           <t>Also implicitly verifies AR-06 auto-forward chain</t>
@@ -6170,12 +6194,16 @@
           <t>accepted_at persists. Status transitions cleanly both ways. Activity log records accept / resolve / reopen with actor + payload.</t>
         </is>
       </c>
-      <c r="G121" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H121" s="5" t="inlineStr"/>
+      <c r="G121" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H121" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I121" s="5" t="inlineStr"/>
     </row>
     <row r="122" ht="60" customHeight="1">
@@ -6210,12 +6238,16 @@
           <t>Upload succeeds. Filename rendered as text everywhere. 5MB cap honoured.</t>
         </is>
       </c>
-      <c r="G122" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H122" s="5" t="inlineStr"/>
+      <c r="G122" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H122" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I122" s="5" t="inlineStr">
         <is>
           <t>CITZ-02 regression on ticket surface</t>
@@ -6255,12 +6287,16 @@
           <t>PDF renders inline (200 OK). Cross-dept access still 403. Prior bug: /department/api/files/ai_uploads/… → 403 for legitimate access.</t>
         </is>
       </c>
-      <c r="G123" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H123" s="5" t="inlineStr"/>
+      <c r="G123" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H123" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I123" s="5" t="inlineStr">
         <is>
           <t>Regression for cbc9c8c (ai_uploads/ branch in _dept_authorize_file) + f40c2f6 (HTTPException import — 500→403 for legit denies)</t>
@@ -6299,12 +6335,16 @@
           <t>Both comments persist with author + timestamp. Tamil no ??? no codec err.</t>
         </is>
       </c>
-      <c r="G124" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H124" s="5" t="inlineStr"/>
+      <c r="G124" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H124" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I124" s="5" t="inlineStr"/>
     </row>
     <row r="125" ht="60" customHeight="1">
@@ -6339,12 +6379,16 @@
           <t>Drawer swaps to sibling row without full-page reload. URL updates. Selection state moves.</t>
         </is>
       </c>
-      <c r="G125" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H125" s="5" t="inlineStr"/>
+      <c r="G125" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H125" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I125" s="5" t="inlineStr"/>
     </row>
     <row r="126" ht="60" customHeight="1">
@@ -6379,12 +6423,16 @@
           <t>pa_admin loads normally. dept_officer redirected or 403 (dept has no association-review UI).</t>
         </is>
       </c>
-      <c r="G126" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H126" s="5" t="inlineStr"/>
+      <c r="G126" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H126" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I126" s="5" t="inlineStr"/>
     </row>
     <row r="127" ht="60" customHeight="1">
@@ -6419,12 +6467,16 @@
           <t>Each tab shows only its status. Empty-state is friendly. Counts match visible rows.</t>
         </is>
       </c>
-      <c r="G127" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H127" s="5" t="inlineStr"/>
+      <c r="G127" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H127" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I127" s="5" t="inlineStr"/>
     </row>
     <row r="128" ht="60" customHeight="1">
@@ -6459,12 +6511,16 @@
           <t>Representative name + phone + org, chosen ministry, AssociationExtraction summary + key details, document previews render inline (iframe).</t>
         </is>
       </c>
-      <c r="G128" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H128" s="5" t="inlineStr"/>
+      <c r="G128" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H128" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I128" s="5" t="inlineStr"/>
     </row>
     <row r="129" ht="60" customHeight="1">
@@ -6500,12 +6556,16 @@
           <t>Ministry edit persists on the row. Approve calls mint_ticket_from_association → Appointment + Ticket + GSR created. Redirect / drawer transitions to 'submitted' state.</t>
         </is>
       </c>
-      <c r="G129" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H129" s="5" t="inlineStr"/>
+      <c r="G129" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H129" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I129" s="5" t="inlineStr">
         <is>
           <t>Regression for 40a6f55 ministry-driven decision refactor</t>
@@ -6544,12 +6604,16 @@
           <t>Ticket exists with status=FORWARDED_TO_DEPT (auto-forwarded via forward_if_non_school). Dept officer can accept from their workspace. SLA fields still editable (see TK-06).</t>
         </is>
       </c>
-      <c r="G130" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H130" s="5" t="inlineStr"/>
+      <c r="G130" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H130" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I130" s="5" t="inlineStr"/>
     </row>
     <row r="131" ht="60" customHeight="1">
@@ -6584,12 +6648,16 @@
           <t>Ticket exists with status=OPEN. Assign panel visible so PA can route to one of the 10 school departments. Contrast with AR-05.</t>
         </is>
       </c>
-      <c r="G131" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H131" s="5" t="inlineStr"/>
+      <c r="G131" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H131" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I131" s="5" t="inlineStr"/>
     </row>
     <row r="132" ht="60" customHeight="1">
@@ -6625,12 +6693,16 @@
           <t>Reason preserved on the row. Restore reverses cleanly. Activity log records both actions.</t>
         </is>
       </c>
-      <c r="G132" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H132" s="5" t="inlineStr"/>
+      <c r="G132" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H132" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I132" s="5" t="inlineStr"/>
     </row>
     <row r="133" ht="60" customHeight="1">
@@ -6665,12 +6737,16 @@
           <t>Every message user-friendly. Zero tracebacks / raw HTTP codes / 'gemini-2.5-flash'. Routed through businessMessage() (errors.ts).</t>
         </is>
       </c>
-      <c r="G133" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H133" s="5" t="inlineStr"/>
+      <c r="G133" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H133" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I133" s="5" t="inlineStr"/>
     </row>
     <row r="134" ht="60" customHeight="1">
@@ -6706,12 +6782,16 @@
           <t>Both drawers scale / go full-screen. All actions reachable with thumbs. No horizontal body scroll.</t>
         </is>
       </c>
-      <c r="G134" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H134" s="5" t="inlineStr"/>
+      <c r="G134" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H134" s="5" t="inlineStr">
+        <is>
+          <t>Verified on Railway</t>
+        </is>
+      </c>
       <c r="I134" s="5" t="inlineStr"/>
     </row>
     <row r="135" ht="60" customHeight="1">

</xml_diff>